<commit_message>
Integration du tableau des cas d'usage auteur dans author[x] de FRLMHeaderDocument 25bce652d3f15caf845501f095686b23295b2466
</commit_message>
<xml_diff>
--- a/fix-target-codes-and-display/ig/StructureDefinition-FRLMHeaderDocument.xlsx
+++ b/fix-target-codes-and-display/ig/StructureDefinition-FRLMHeaderDocument.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="138">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-25T11:56:50+00:00</t>
+    <t>2026-08-25T20:08:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -342,6 +342,17 @@
   </si>
   <si>
     <t>Auteur du document.</t>
+  </si>
+  <si>
+    <t>Voici les cas d'usage des documents et leurs auteurs :
+| Cas d'usage | Auteur(s) du document | Structure de l'auteur |
+|-------------|----------------------|-----------------------|
+| Création d'un document par un professionnel sur son logiciel professionnel | Professionnel | Structure |
+| Création d'un document patient par un professionnel sur son logiciel professionnel pour le compte du patient | Professionnel | Structure |
+| Création d'un document patient par le patient | Patient | non utilisé |
+| Création d'un document par un système (dispositif, automate, …) de structure (ES, …) | Système de structure | Structure |
+| Création d'un document par un Service numérique référencé (SNR) | SNR | Editeur |
+| Création d'un document par le DP | CNOP/DP | CNOP |</t>
   </si>
   <si>
     <t>FRLMHeaderDocument.dataEnterer</t>
@@ -2029,7 +2040,9 @@
       <c r="M13" t="s" s="2">
         <v>106</v>
       </c>
-      <c r="N13" s="2"/>
+      <c r="N13" t="s" s="2">
+        <v>107</v>
+      </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
         <v>72</v>
@@ -2095,10 +2108,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2121,13 +2134,13 @@
         <v>72</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2178,7 +2191,7 @@
         <v>72</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>73</v>
@@ -2195,10 +2208,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2221,13 +2234,13 @@
         <v>72</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2278,7 +2291,7 @@
         <v>72</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>73</v>
@@ -2295,10 +2308,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2321,13 +2334,13 @@
         <v>72</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2378,7 +2391,7 @@
         <v>72</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>78</v>
@@ -2395,10 +2408,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2421,13 +2434,13 @@
         <v>72</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2478,7 +2491,7 @@
         <v>72</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>73</v>
@@ -2495,10 +2508,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2521,13 +2534,13 @@
         <v>72</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -2578,7 +2591,7 @@
         <v>72</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>78</v>
@@ -2595,10 +2608,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2621,13 +2634,13 @@
         <v>72</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2678,7 +2691,7 @@
         <v>72</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>73</v>
@@ -2695,10 +2708,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2721,13 +2734,13 @@
         <v>72</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2778,7 +2791,7 @@
         <v>72</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>73</v>
@@ -2795,10 +2808,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2821,13 +2834,13 @@
         <v>72</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -2878,7 +2891,7 @@
         <v>72</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>73</v>
@@ -2895,10 +2908,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -2921,13 +2934,13 @@
         <v>72</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -2978,7 +2991,7 @@
         <v>72</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>73</v>
@@ -2995,10 +3008,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3021,13 +3034,13 @@
         <v>72</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3078,7 +3091,7 @@
         <v>72</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>

</xml_diff>